<commit_message>
v1.1.0: PDF output, milestones on the Gantt, robust HTML preview, first-person README
</commit_message>
<xml_diff>
--- a/assets/sample-outputs/sample-project-plan.xlsx
+++ b/assets/sample-outputs/sample-project-plan.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="25">
+  <fonts count="30">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -125,6 +125,36 @@
       <name val="Calibri"/>
       <color rgb="004A4A4A"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="003F7A52"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="003F7A52"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00AE7A2A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00AE7A2A"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00081A30"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -259,7 +289,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -299,44 +329,59 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="18" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="23" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -413,6 +458,61 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Project Plan Generator</author>
+  </authors>
+  <commentList>
+    <comment ref="I9" authorId="0" shapeId="0">
+      <text>
+        <t>Concept design approved — 27 March 2026 (Achieved)</t>
+      </text>
+    </comment>
+    <comment ref="L10" authorId="0" shapeId="0">
+      <text>
+        <t>Detailed design sign-off — 17 April 2026 (Achieved)</t>
+      </text>
+    </comment>
+    <comment ref="N11" authorId="0" shapeId="0">
+      <text>
+        <t>Permits approved — 30 April 2026 (At risk)</t>
+      </text>
+    </comment>
+    <comment ref="N12" authorId="0" shapeId="0">
+      <text>
+        <t>Contractor appointed — 01 May 2026 (On track)</t>
+      </text>
+    </comment>
+    <comment ref="O13" authorId="0" shapeId="0">
+      <text>
+        <t>Site handover — 08 May 2026 (On track)</t>
+      </text>
+    </comment>
+    <comment ref="U14" authorId="0" shapeId="0">
+      <text>
+        <t>Structural alterations complete — 19 June 2026 (On track)</t>
+      </text>
+    </comment>
+    <comment ref="Z15" authorId="0" shapeId="0">
+      <text>
+        <t>MEP first fix complete — 24 July 2026 (On track)</t>
+      </text>
+    </comment>
+    <comment ref="AH16" authorId="0" shapeId="0">
+      <text>
+        <t>Practical completion — 15 September 2026 (On track)</t>
+      </text>
+    </comment>
+    <comment ref="AI17" authorId="0" shapeId="0">
+      <text>
+        <t>Handover to client — 25 September 2026 (On track)</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -960,7 +1060,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AI25"/>
+  <dimension ref="B2:AI35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1234,421 +1334,684 @@
     <row r="8" ht="22" customHeight="1">
       <c r="B8" s="22" t="inlineStr">
         <is>
-          <t>DESIGN &amp; PERMITS</t>
+          <t>MILESTONES</t>
         </is>
       </c>
       <c r="C8" s="23" t="n"/>
       <c r="D8" s="23" t="n"/>
       <c r="E8" s="23" t="n"/>
-      <c r="F8" s="24" t="n"/>
-      <c r="G8" s="24" t="n"/>
-      <c r="H8" s="24" t="n"/>
-      <c r="I8" s="24" t="n"/>
-      <c r="J8" s="24" t="n"/>
-      <c r="K8" s="24" t="n"/>
-      <c r="L8" s="25" t="n"/>
-      <c r="M8" s="24" t="n"/>
-      <c r="N8" s="24" t="n"/>
+      <c r="L8" s="24" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Programme &amp; brief</t>
-        </is>
-      </c>
-      <c r="C9" s="26" t="inlineStr">
-        <is>
-          <t>PM</t>
-        </is>
-      </c>
-      <c r="D9" s="26" t="inlineStr">
-        <is>
-          <t>02 Mar</t>
-        </is>
-      </c>
-      <c r="E9" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" s="28" t="n"/>
-      <c r="G9" s="28" t="n"/>
-      <c r="L9" s="29" t="n"/>
+          <t xml:space="preserve">  ◆ Concept design approved</t>
+        </is>
+      </c>
+      <c r="C9" s="25" t="inlineStr">
+        <is>
+          <t>Architect</t>
+        </is>
+      </c>
+      <c r="D9" s="25" t="inlineStr">
+        <is>
+          <t>27 Mar</t>
+        </is>
+      </c>
+      <c r="E9" s="26" t="inlineStr">
+        <is>
+          <t>Achieved</t>
+        </is>
+      </c>
+      <c r="I9" s="27" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
+      <c r="L9" s="24" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Concept design</t>
-        </is>
-      </c>
-      <c r="C10" s="26" t="inlineStr">
+          <t xml:space="preserve">  ◆ Detailed design sign-off</t>
+        </is>
+      </c>
+      <c r="C10" s="25" t="inlineStr">
         <is>
           <t>Architect</t>
         </is>
       </c>
-      <c r="D10" s="26" t="inlineStr">
-        <is>
-          <t>16 Mar</t>
-        </is>
-      </c>
-      <c r="E10" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" s="28" t="n"/>
-      <c r="I10" s="28" t="n"/>
-      <c r="L10" s="29" t="n"/>
+      <c r="D10" s="25" t="inlineStr">
+        <is>
+          <t>17 Apr</t>
+        </is>
+      </c>
+      <c r="E10" s="26" t="inlineStr">
+        <is>
+          <t>Achieved</t>
+        </is>
+      </c>
+      <c r="L10" s="28" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Detailed design</t>
-        </is>
-      </c>
-      <c r="C11" s="26" t="inlineStr">
-        <is>
-          <t>Architect</t>
-        </is>
-      </c>
-      <c r="D11" s="26" t="inlineStr">
-        <is>
-          <t>30 Mar</t>
-        </is>
-      </c>
-      <c r="E11" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="J11" s="28" t="n"/>
-      <c r="K11" s="28" t="n"/>
-      <c r="L11" s="30" t="n"/>
+          <t xml:space="preserve">  ◆ Permits approved</t>
+        </is>
+      </c>
+      <c r="C11" s="25" t="inlineStr">
+        <is>
+          <t>Permit Consultant</t>
+        </is>
+      </c>
+      <c r="D11" s="25" t="inlineStr">
+        <is>
+          <t>30 Apr</t>
+        </is>
+      </c>
+      <c r="E11" s="29" t="inlineStr">
+        <is>
+          <t>At risk</t>
+        </is>
+      </c>
+      <c r="L11" s="24" t="n"/>
+      <c r="N11" s="30" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Permit applications</t>
-        </is>
-      </c>
-      <c r="C12" s="26" t="inlineStr">
-        <is>
-          <t>Permit Consultant</t>
-        </is>
-      </c>
-      <c r="D12" s="26" t="inlineStr">
-        <is>
-          <t>06 Apr</t>
-        </is>
-      </c>
-      <c r="E12" s="27" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="K12" s="31" t="n"/>
-      <c r="L12" s="32" t="n"/>
-      <c r="M12" s="33" t="n"/>
-      <c r="N12" s="33" t="n"/>
+          <t xml:space="preserve">  ◆ Contractor appointed</t>
+        </is>
+      </c>
+      <c r="C12" s="25" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="D12" s="25" t="inlineStr">
+        <is>
+          <t>01 May</t>
+        </is>
+      </c>
+      <c r="E12" s="31" t="inlineStr">
+        <is>
+          <t>On track</t>
+        </is>
+      </c>
+      <c r="L12" s="24" t="n"/>
+      <c r="N12" s="32" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Tender &amp; contractor selection</t>
-        </is>
-      </c>
-      <c r="C13" s="26" t="inlineStr">
-        <is>
-          <t>PM</t>
-        </is>
-      </c>
-      <c r="D13" s="26" t="inlineStr">
-        <is>
-          <t>13 Apr</t>
-        </is>
-      </c>
-      <c r="E13" s="27" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="L13" s="32" t="n"/>
-      <c r="M13" s="24" t="n"/>
-      <c r="N13" s="24" t="n"/>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="22" t="inlineStr">
-        <is>
-          <t>DEMOLITION &amp; STRUCTURAL</t>
-        </is>
-      </c>
-      <c r="C14" s="23" t="n"/>
-      <c r="D14" s="23" t="n"/>
-      <c r="E14" s="23" t="n"/>
-      <c r="L14" s="29" t="n"/>
-      <c r="O14" s="24" t="n"/>
-      <c r="P14" s="24" t="n"/>
-      <c r="Q14" s="24" t="n"/>
-      <c r="R14" s="24" t="n"/>
-      <c r="S14" s="24" t="n"/>
-      <c r="T14" s="24" t="n"/>
-      <c r="U14" s="24" t="n"/>
+          <t xml:space="preserve">  ◆ Site handover</t>
+        </is>
+      </c>
+      <c r="C13" s="25" t="inlineStr">
+        <is>
+          <t>Contractor</t>
+        </is>
+      </c>
+      <c r="D13" s="25" t="inlineStr">
+        <is>
+          <t>08 May</t>
+        </is>
+      </c>
+      <c r="E13" s="31" t="inlineStr">
+        <is>
+          <t>On track</t>
+        </is>
+      </c>
+      <c r="L13" s="24" t="n"/>
+      <c r="O13" s="32" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ◆ Structural alterations complete</t>
+        </is>
+      </c>
+      <c r="C14" s="25" t="inlineStr">
+        <is>
+          <t>Structural Engineer</t>
+        </is>
+      </c>
+      <c r="D14" s="25" t="inlineStr">
+        <is>
+          <t>19 Jun</t>
+        </is>
+      </c>
+      <c r="E14" s="31" t="inlineStr">
+        <is>
+          <t>On track</t>
+        </is>
+      </c>
+      <c r="L14" s="24" t="n"/>
+      <c r="U14" s="32" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Site handover &amp; mobilisation</t>
-        </is>
-      </c>
-      <c r="C15" s="26" t="inlineStr">
+          <t xml:space="preserve">  ◆ MEP first fix complete</t>
+        </is>
+      </c>
+      <c r="C15" s="25" t="inlineStr">
         <is>
           <t>Contractor</t>
         </is>
       </c>
-      <c r="D15" s="26" t="inlineStr">
-        <is>
-          <t>04 May</t>
-        </is>
-      </c>
-      <c r="E15" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" s="29" t="n"/>
-      <c r="O15" s="24" t="n"/>
+      <c r="D15" s="25" t="inlineStr">
+        <is>
+          <t>24 Jul</t>
+        </is>
+      </c>
+      <c r="E15" s="31" t="inlineStr">
+        <is>
+          <t>On track</t>
+        </is>
+      </c>
+      <c r="L15" s="24" t="n"/>
+      <c r="Z15" s="32" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Demolition</t>
-        </is>
-      </c>
-      <c r="C16" s="26" t="inlineStr">
-        <is>
-          <t>Contractor</t>
-        </is>
-      </c>
-      <c r="D16" s="26" t="inlineStr">
-        <is>
-          <t>11 May</t>
-        </is>
-      </c>
-      <c r="E16" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" s="29" t="n"/>
-      <c r="P16" s="24" t="n"/>
-      <c r="Q16" s="24" t="n"/>
-      <c r="R16" s="24" t="n"/>
+          <t xml:space="preserve">  ◆ Practical completion</t>
+        </is>
+      </c>
+      <c r="C16" s="25" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="D16" s="25" t="inlineStr">
+        <is>
+          <t>15 Sep</t>
+        </is>
+      </c>
+      <c r="E16" s="31" t="inlineStr">
+        <is>
+          <t>On track</t>
+        </is>
+      </c>
+      <c r="L16" s="24" t="n"/>
+      <c r="AH16" s="32" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Structural alterations</t>
-        </is>
-      </c>
-      <c r="C17" s="26" t="inlineStr">
-        <is>
-          <t>Structural Engineer</t>
-        </is>
-      </c>
-      <c r="D17" s="26" t="inlineStr">
-        <is>
-          <t>01 Jun</t>
-        </is>
-      </c>
-      <c r="E17" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" s="29" t="n"/>
-      <c r="S17" s="24" t="n"/>
-      <c r="T17" s="24" t="n"/>
-      <c r="U17" s="24" t="n"/>
+          <t xml:space="preserve">  ◆ Handover to client</t>
+        </is>
+      </c>
+      <c r="C17" s="25" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="D17" s="25" t="inlineStr">
+        <is>
+          <t>25 Sep</t>
+        </is>
+      </c>
+      <c r="E17" s="31" t="inlineStr">
+        <is>
+          <t>On track</t>
+        </is>
+      </c>
+      <c r="L17" s="24" t="n"/>
+      <c r="AI17" s="32" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="B18" s="22" t="inlineStr">
         <is>
-          <t>FIT-OUT &amp; SERVICES</t>
+          <t>DESIGN &amp; PERMITS</t>
         </is>
       </c>
       <c r="C18" s="23" t="n"/>
       <c r="D18" s="23" t="n"/>
       <c r="E18" s="23" t="n"/>
-      <c r="L18" s="29" t="n"/>
-      <c r="V18" s="24" t="n"/>
-      <c r="W18" s="24" t="n"/>
-      <c r="X18" s="24" t="n"/>
-      <c r="Y18" s="24" t="n"/>
-      <c r="Z18" s="24" t="n"/>
-      <c r="AA18" s="24" t="n"/>
-      <c r="AB18" s="24" t="n"/>
-      <c r="AC18" s="24" t="n"/>
-      <c r="AD18" s="24" t="n"/>
-      <c r="AE18" s="24" t="n"/>
+      <c r="F18" s="33" t="n"/>
+      <c r="G18" s="33" t="n"/>
+      <c r="H18" s="33" t="n"/>
+      <c r="I18" s="33" t="n"/>
+      <c r="J18" s="33" t="n"/>
+      <c r="K18" s="33" t="n"/>
+      <c r="L18" s="34" t="n"/>
+      <c r="M18" s="33" t="n"/>
+      <c r="N18" s="33" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MEP first fix</t>
-        </is>
-      </c>
-      <c r="C19" s="26" t="inlineStr">
-        <is>
-          <t>Contractor</t>
-        </is>
-      </c>
-      <c r="D19" s="26" t="inlineStr">
-        <is>
-          <t>22 Jun</t>
-        </is>
-      </c>
-      <c r="E19" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" s="29" t="n"/>
-      <c r="V19" s="24" t="n"/>
-      <c r="W19" s="24" t="n"/>
-      <c r="X19" s="24" t="n"/>
-      <c r="Y19" s="24" t="n"/>
-      <c r="Z19" s="24" t="n"/>
+          <t xml:space="preserve">  Programme &amp; brief</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="D19" s="25" t="inlineStr">
+        <is>
+          <t>02 Mar</t>
+        </is>
+      </c>
+      <c r="E19" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="36" t="n"/>
+      <c r="G19" s="36" t="n"/>
+      <c r="L19" s="24" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Partitions &amp; ceilings</t>
-        </is>
-      </c>
-      <c r="C20" s="26" t="inlineStr">
-        <is>
-          <t>Contractor</t>
-        </is>
-      </c>
-      <c r="D20" s="26" t="inlineStr">
-        <is>
-          <t>13 Jul</t>
-        </is>
-      </c>
-      <c r="E20" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" s="29" t="n"/>
-      <c r="Y20" s="24" t="n"/>
-      <c r="Z20" s="24" t="n"/>
-      <c r="AA20" s="24" t="n"/>
-      <c r="AB20" s="24" t="n"/>
+          <t xml:space="preserve">  Concept design</t>
+        </is>
+      </c>
+      <c r="C20" s="25" t="inlineStr">
+        <is>
+          <t>Architect</t>
+        </is>
+      </c>
+      <c r="D20" s="25" t="inlineStr">
+        <is>
+          <t>16 Mar</t>
+        </is>
+      </c>
+      <c r="E20" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="36" t="n"/>
+      <c r="I20" s="36" t="n"/>
+      <c r="L20" s="24" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Finishes</t>
-        </is>
-      </c>
-      <c r="C21" s="26" t="inlineStr">
-        <is>
-          <t>Contractor</t>
-        </is>
-      </c>
-      <c r="D21" s="26" t="inlineStr">
-        <is>
-          <t>03 Aug</t>
-        </is>
-      </c>
-      <c r="E21" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" s="29" t="n"/>
-      <c r="AB21" s="24" t="n"/>
-      <c r="AC21" s="24" t="n"/>
-      <c r="AD21" s="24" t="n"/>
+          <t xml:space="preserve">  Detailed design</t>
+        </is>
+      </c>
+      <c r="C21" s="25" t="inlineStr">
+        <is>
+          <t>Architect</t>
+        </is>
+      </c>
+      <c r="D21" s="25" t="inlineStr">
+        <is>
+          <t>30 Mar</t>
+        </is>
+      </c>
+      <c r="E21" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" s="36" t="n"/>
+      <c r="K21" s="36" t="n"/>
+      <c r="L21" s="37" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="B22" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FF&amp;E installation</t>
-        </is>
-      </c>
-      <c r="C22" s="26" t="inlineStr">
-        <is>
-          <t>FF&amp;E Supplier</t>
-        </is>
-      </c>
-      <c r="D22" s="26" t="inlineStr">
-        <is>
-          <t>17 Aug</t>
-        </is>
-      </c>
-      <c r="E22" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" s="29" t="n"/>
-      <c r="AD22" s="24" t="n"/>
-      <c r="AE22" s="24" t="n"/>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="B23" s="22" t="inlineStr">
-        <is>
-          <t>SNAGGING &amp; HANDOVER</t>
-        </is>
-      </c>
-      <c r="C23" s="23" t="n"/>
-      <c r="D23" s="23" t="n"/>
-      <c r="E23" s="23" t="n"/>
-      <c r="L23" s="29" t="n"/>
-      <c r="AF23" s="24" t="n"/>
-      <c r="AG23" s="24" t="n"/>
-      <c r="AH23" s="24" t="n"/>
-      <c r="AI23" s="24" t="n"/>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="B24" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Commissioning</t>
-        </is>
-      </c>
-      <c r="C24" s="26" t="inlineStr">
-        <is>
-          <t>Contractor</t>
-        </is>
-      </c>
-      <c r="D24" s="26" t="inlineStr">
-        <is>
-          <t>31 Aug</t>
-        </is>
-      </c>
-      <c r="E24" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" s="29" t="n"/>
-      <c r="AF24" s="24" t="n"/>
-      <c r="AG24" s="24" t="n"/>
+          <t xml:space="preserve">  Permit applications</t>
+        </is>
+      </c>
+      <c r="C22" s="25" t="inlineStr">
+        <is>
+          <t>Permit Consultant</t>
+        </is>
+      </c>
+      <c r="D22" s="25" t="inlineStr">
+        <is>
+          <t>06 Apr</t>
+        </is>
+      </c>
+      <c r="E22" s="35" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="K22" s="38" t="n"/>
+      <c r="L22" s="39" t="n"/>
+      <c r="M22" s="40" t="n"/>
+      <c r="N22" s="40" t="n"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Tender &amp; contractor selection</t>
+        </is>
+      </c>
+      <c r="C23" s="25" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="D23" s="25" t="inlineStr">
+        <is>
+          <t>13 Apr</t>
+        </is>
+      </c>
+      <c r="E23" s="35" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="L23" s="39" t="n"/>
+      <c r="M23" s="33" t="n"/>
+      <c r="N23" s="33" t="n"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="B24" s="22" t="inlineStr">
+        <is>
+          <t>DEMOLITION &amp; STRUCTURAL</t>
+        </is>
+      </c>
+      <c r="C24" s="23" t="n"/>
+      <c r="D24" s="23" t="n"/>
+      <c r="E24" s="23" t="n"/>
+      <c r="L24" s="24" t="n"/>
+      <c r="O24" s="33" t="n"/>
+      <c r="P24" s="33" t="n"/>
+      <c r="Q24" s="33" t="n"/>
+      <c r="R24" s="33" t="n"/>
+      <c r="S24" s="33" t="n"/>
+      <c r="T24" s="33" t="n"/>
+      <c r="U24" s="33" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="B25" s="13" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Site handover &amp; mobilisation</t>
+        </is>
+      </c>
+      <c r="C25" s="25" t="inlineStr">
+        <is>
+          <t>Contractor</t>
+        </is>
+      </c>
+      <c r="D25" s="25" t="inlineStr">
+        <is>
+          <t>04 May</t>
+        </is>
+      </c>
+      <c r="E25" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="24" t="n"/>
+      <c r="O25" s="33" t="n"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Demolition</t>
+        </is>
+      </c>
+      <c r="C26" s="25" t="inlineStr">
+        <is>
+          <t>Contractor</t>
+        </is>
+      </c>
+      <c r="D26" s="25" t="inlineStr">
+        <is>
+          <t>11 May</t>
+        </is>
+      </c>
+      <c r="E26" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="24" t="n"/>
+      <c r="P26" s="33" t="n"/>
+      <c r="Q26" s="33" t="n"/>
+      <c r="R26" s="33" t="n"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Structural alterations</t>
+        </is>
+      </c>
+      <c r="C27" s="25" t="inlineStr">
+        <is>
+          <t>Structural Engineer</t>
+        </is>
+      </c>
+      <c r="D27" s="25" t="inlineStr">
+        <is>
+          <t>01 Jun</t>
+        </is>
+      </c>
+      <c r="E27" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="24" t="n"/>
+      <c r="S27" s="33" t="n"/>
+      <c r="T27" s="33" t="n"/>
+      <c r="U27" s="33" t="n"/>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="B28" s="22" t="inlineStr">
+        <is>
+          <t>FIT-OUT &amp; SERVICES</t>
+        </is>
+      </c>
+      <c r="C28" s="23" t="n"/>
+      <c r="D28" s="23" t="n"/>
+      <c r="E28" s="23" t="n"/>
+      <c r="L28" s="24" t="n"/>
+      <c r="V28" s="33" t="n"/>
+      <c r="W28" s="33" t="n"/>
+      <c r="X28" s="33" t="n"/>
+      <c r="Y28" s="33" t="n"/>
+      <c r="Z28" s="33" t="n"/>
+      <c r="AA28" s="33" t="n"/>
+      <c r="AB28" s="33" t="n"/>
+      <c r="AC28" s="33" t="n"/>
+      <c r="AD28" s="33" t="n"/>
+      <c r="AE28" s="33" t="n"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MEP first fix</t>
+        </is>
+      </c>
+      <c r="C29" s="25" t="inlineStr">
+        <is>
+          <t>Contractor</t>
+        </is>
+      </c>
+      <c r="D29" s="25" t="inlineStr">
+        <is>
+          <t>22 Jun</t>
+        </is>
+      </c>
+      <c r="E29" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="24" t="n"/>
+      <c r="V29" s="33" t="n"/>
+      <c r="W29" s="33" t="n"/>
+      <c r="X29" s="33" t="n"/>
+      <c r="Y29" s="33" t="n"/>
+      <c r="Z29" s="33" t="n"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Partitions &amp; ceilings</t>
+        </is>
+      </c>
+      <c r="C30" s="25" t="inlineStr">
+        <is>
+          <t>Contractor</t>
+        </is>
+      </c>
+      <c r="D30" s="25" t="inlineStr">
+        <is>
+          <t>13 Jul</t>
+        </is>
+      </c>
+      <c r="E30" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="24" t="n"/>
+      <c r="Y30" s="33" t="n"/>
+      <c r="Z30" s="33" t="n"/>
+      <c r="AA30" s="33" t="n"/>
+      <c r="AB30" s="33" t="n"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Finishes</t>
+        </is>
+      </c>
+      <c r="C31" s="25" t="inlineStr">
+        <is>
+          <t>Contractor</t>
+        </is>
+      </c>
+      <c r="D31" s="25" t="inlineStr">
+        <is>
+          <t>03 Aug</t>
+        </is>
+      </c>
+      <c r="E31" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" s="24" t="n"/>
+      <c r="AB31" s="33" t="n"/>
+      <c r="AC31" s="33" t="n"/>
+      <c r="AD31" s="33" t="n"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  FF&amp;E installation</t>
+        </is>
+      </c>
+      <c r="C32" s="25" t="inlineStr">
+        <is>
+          <t>FF&amp;E Supplier</t>
+        </is>
+      </c>
+      <c r="D32" s="25" t="inlineStr">
+        <is>
+          <t>17 Aug</t>
+        </is>
+      </c>
+      <c r="E32" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" s="24" t="n"/>
+      <c r="AD32" s="33" t="n"/>
+      <c r="AE32" s="33" t="n"/>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="B33" s="22" t="inlineStr">
+        <is>
+          <t>SNAGGING &amp; HANDOVER</t>
+        </is>
+      </c>
+      <c r="C33" s="23" t="n"/>
+      <c r="D33" s="23" t="n"/>
+      <c r="E33" s="23" t="n"/>
+      <c r="L33" s="24" t="n"/>
+      <c r="AF33" s="33" t="n"/>
+      <c r="AG33" s="33" t="n"/>
+      <c r="AH33" s="33" t="n"/>
+      <c r="AI33" s="33" t="n"/>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Commissioning</t>
+        </is>
+      </c>
+      <c r="C34" s="25" t="inlineStr">
+        <is>
+          <t>Contractor</t>
+        </is>
+      </c>
+      <c r="D34" s="25" t="inlineStr">
+        <is>
+          <t>31 Aug</t>
+        </is>
+      </c>
+      <c r="E34" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="24" t="n"/>
+      <c r="AF34" s="33" t="n"/>
+      <c r="AG34" s="33" t="n"/>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="B35" s="13" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Snagging &amp; client sign-off</t>
         </is>
       </c>
-      <c r="C25" s="26" t="inlineStr">
+      <c r="C35" s="25" t="inlineStr">
         <is>
           <t>PM</t>
         </is>
       </c>
-      <c r="D25" s="26" t="inlineStr">
+      <c r="D35" s="25" t="inlineStr">
         <is>
           <t>14 Sep</t>
         </is>
       </c>
-      <c r="E25" s="27" t="n">
+      <c r="E35" s="35" t="n">
         <v>0</v>
       </c>
-      <c r="L25" s="29" t="n"/>
-      <c r="AH25" s="24" t="n"/>
-      <c r="AI25" s="24" t="n"/>
+      <c r="L35" s="24" t="n"/>
+      <c r="AH35" s="33" t="n"/>
+      <c r="AI35" s="33" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="B23:E23"/>
+  <mergeCells count="12">
     <mergeCell ref="K6:N6"/>
     <mergeCell ref="B18:E18"/>
     <mergeCell ref="B8:E8"/>
     <mergeCell ref="AB6:AF6"/>
     <mergeCell ref="X6:AA6"/>
+    <mergeCell ref="B33:E33"/>
     <mergeCell ref="S6:W6"/>
+    <mergeCell ref="B24:E24"/>
     <mergeCell ref="F6:J6"/>
     <mergeCell ref="O6:R6"/>
+    <mergeCell ref="B28:E28"/>
     <mergeCell ref="AG6:AI6"/>
-    <mergeCell ref="B14:E14"/>
   </mergeCells>
-  <conditionalFormatting sqref="E9:E13">
+  <conditionalFormatting sqref="E19:E23">
     <cfRule type="dataBar" priority="1">
       <dataBar showValue="1">
         <cfvo type="num" val="0"/>
@@ -1657,7 +2020,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E15:E17">
+  <conditionalFormatting sqref="E25:E27">
     <cfRule type="dataBar" priority="2">
       <dataBar showValue="1">
         <cfvo type="num" val="0"/>
@@ -1666,7 +2029,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E19:E22">
+  <conditionalFormatting sqref="E29:E32">
     <cfRule type="dataBar" priority="3">
       <dataBar showValue="1">
         <cfvo type="num" val="0"/>
@@ -1675,7 +2038,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E24:E25">
+  <conditionalFormatting sqref="E34:E35">
     <cfRule type="dataBar" priority="4">
       <dataBar showValue="1">
         <cfvo type="num" val="0"/>
@@ -1685,6 +2048,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1760,288 +2124,288 @@
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
-      <c r="B7" s="34" t="inlineStr">
+      <c r="B7" s="41" t="inlineStr">
         <is>
           <t>M01</t>
         </is>
       </c>
-      <c r="C7" s="35" t="inlineStr">
+      <c r="C7" s="42" t="inlineStr">
         <is>
           <t>Concept design approved</t>
         </is>
       </c>
-      <c r="D7" s="36" t="inlineStr">
+      <c r="D7" s="43" t="inlineStr">
         <is>
           <t>27 Mar 2026</t>
         </is>
       </c>
-      <c r="E7" s="37" t="inlineStr">
+      <c r="E7" s="44" t="inlineStr">
         <is>
           <t>Achieved</t>
         </is>
       </c>
-      <c r="F7" s="38" t="inlineStr">
+      <c r="F7" s="45" t="inlineStr">
         <is>
           <t>Architect</t>
         </is>
       </c>
-      <c r="G7" s="39" t="inlineStr">
+      <c r="G7" s="46" t="inlineStr">
         <is>
           <t>Client signed off the concept design and footprint.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
-      <c r="B8" s="34" t="inlineStr">
+      <c r="B8" s="41" t="inlineStr">
         <is>
           <t>M02</t>
         </is>
       </c>
-      <c r="C8" s="35" t="inlineStr">
+      <c r="C8" s="42" t="inlineStr">
         <is>
           <t>Detailed design sign-off</t>
         </is>
       </c>
-      <c r="D8" s="36" t="inlineStr">
+      <c r="D8" s="43" t="inlineStr">
         <is>
           <t>17 Apr 2026</t>
         </is>
       </c>
-      <c r="E8" s="37" t="inlineStr">
+      <c r="E8" s="44" t="inlineStr">
         <is>
           <t>Achieved</t>
         </is>
       </c>
-      <c r="F8" s="38" t="inlineStr">
+      <c r="F8" s="45" t="inlineStr">
         <is>
           <t>Architect</t>
         </is>
       </c>
-      <c r="G8" s="39" t="inlineStr">
+      <c r="G8" s="46" t="inlineStr">
         <is>
           <t>Detailed drawings, spec, and FF&amp;E schedule approved.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
-      <c r="B9" s="34" t="inlineStr">
+      <c r="B9" s="41" t="inlineStr">
         <is>
           <t>M03</t>
         </is>
       </c>
-      <c r="C9" s="35" t="inlineStr">
+      <c r="C9" s="42" t="inlineStr">
         <is>
           <t>Permits approved</t>
         </is>
       </c>
-      <c r="D9" s="36" t="inlineStr">
+      <c r="D9" s="43" t="inlineStr">
         <is>
           <t>30 Apr 2026</t>
         </is>
       </c>
-      <c r="E9" s="40" t="inlineStr">
+      <c r="E9" s="47" t="inlineStr">
         <is>
           <t>At risk</t>
         </is>
       </c>
-      <c r="F9" s="38" t="inlineStr">
+      <c r="F9" s="45" t="inlineStr">
         <is>
           <t>Permit Consultant</t>
         </is>
       </c>
-      <c r="G9" s="39" t="inlineStr">
+      <c r="G9" s="46" t="inlineStr">
         <is>
           <t>City sign-off on building and mechanical permits. Currently five working days behind the target date.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
-      <c r="B10" s="34" t="inlineStr">
+      <c r="B10" s="41" t="inlineStr">
         <is>
           <t>M04</t>
         </is>
       </c>
-      <c r="C10" s="35" t="inlineStr">
+      <c r="C10" s="42" t="inlineStr">
         <is>
           <t>Contractor appointed</t>
         </is>
       </c>
-      <c r="D10" s="36" t="inlineStr">
+      <c r="D10" s="43" t="inlineStr">
         <is>
           <t>01 May 2026</t>
         </is>
       </c>
-      <c r="E10" s="41" t="inlineStr">
+      <c r="E10" s="48" t="inlineStr">
         <is>
           <t>On track</t>
         </is>
       </c>
-      <c r="F10" s="38" t="inlineStr">
+      <c r="F10" s="45" t="inlineStr">
         <is>
           <t>PM</t>
         </is>
       </c>
-      <c r="G10" s="39" t="inlineStr">
+      <c r="G10" s="46" t="inlineStr">
         <is>
           <t>Signed main contract with preferred contractor.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1">
-      <c r="B11" s="34" t="inlineStr">
+      <c r="B11" s="41" t="inlineStr">
         <is>
           <t>M05</t>
         </is>
       </c>
-      <c r="C11" s="35" t="inlineStr">
+      <c r="C11" s="42" t="inlineStr">
         <is>
           <t>Site handover</t>
         </is>
       </c>
-      <c r="D11" s="36" t="inlineStr">
+      <c r="D11" s="43" t="inlineStr">
         <is>
           <t>08 May 2026</t>
         </is>
       </c>
-      <c r="E11" s="41" t="inlineStr">
+      <c r="E11" s="48" t="inlineStr">
         <is>
           <t>On track</t>
         </is>
       </c>
-      <c r="F11" s="38" t="inlineStr">
+      <c r="F11" s="45" t="inlineStr">
         <is>
           <t>Contractor</t>
         </is>
       </c>
-      <c r="G11" s="39" t="inlineStr">
+      <c r="G11" s="46" t="inlineStr">
         <is>
           <t>Physical handover of the building to the main contractor for works.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
-      <c r="B12" s="34" t="inlineStr">
+      <c r="B12" s="41" t="inlineStr">
         <is>
           <t>M06</t>
         </is>
       </c>
-      <c r="C12" s="35" t="inlineStr">
+      <c r="C12" s="42" t="inlineStr">
         <is>
           <t>Structural alterations complete</t>
         </is>
       </c>
-      <c r="D12" s="36" t="inlineStr">
+      <c r="D12" s="43" t="inlineStr">
         <is>
           <t>19 Jun 2026</t>
         </is>
       </c>
-      <c r="E12" s="41" t="inlineStr">
+      <c r="E12" s="48" t="inlineStr">
         <is>
           <t>On track</t>
         </is>
       </c>
-      <c r="F12" s="38" t="inlineStr">
+      <c r="F12" s="45" t="inlineStr">
         <is>
           <t>Structural Engineer</t>
         </is>
       </c>
-      <c r="G12" s="39" t="inlineStr">
+      <c r="G12" s="46" t="inlineStr">
         <is>
           <t>All demolition and structural changes signed off by the engineer.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1">
-      <c r="B13" s="34" t="inlineStr">
+      <c r="B13" s="41" t="inlineStr">
         <is>
           <t>M07</t>
         </is>
       </c>
-      <c r="C13" s="35" t="inlineStr">
+      <c r="C13" s="42" t="inlineStr">
         <is>
           <t>MEP first fix complete</t>
         </is>
       </c>
-      <c r="D13" s="36" t="inlineStr">
+      <c r="D13" s="43" t="inlineStr">
         <is>
           <t>24 Jul 2026</t>
         </is>
       </c>
-      <c r="E13" s="41" t="inlineStr">
+      <c r="E13" s="48" t="inlineStr">
         <is>
           <t>On track</t>
         </is>
       </c>
-      <c r="F13" s="38" t="inlineStr">
+      <c r="F13" s="45" t="inlineStr">
         <is>
           <t>Contractor</t>
         </is>
       </c>
-      <c r="G13" s="39" t="inlineStr">
+      <c r="G13" s="46" t="inlineStr">
         <is>
           <t>Mechanical, electrical, and plumbing first fix signed off.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1">
-      <c r="B14" s="34" t="inlineStr">
+      <c r="B14" s="41" t="inlineStr">
         <is>
           <t>M08</t>
         </is>
       </c>
-      <c r="C14" s="35" t="inlineStr">
+      <c r="C14" s="42" t="inlineStr">
         <is>
           <t>Practical completion</t>
         </is>
       </c>
-      <c r="D14" s="36" t="inlineStr">
+      <c r="D14" s="43" t="inlineStr">
         <is>
           <t>15 Sep 2026</t>
         </is>
       </c>
-      <c r="E14" s="41" t="inlineStr">
+      <c r="E14" s="48" t="inlineStr">
         <is>
           <t>On track</t>
         </is>
       </c>
-      <c r="F14" s="38" t="inlineStr">
+      <c r="F14" s="45" t="inlineStr">
         <is>
           <t>PM</t>
         </is>
       </c>
-      <c r="G14" s="39" t="inlineStr">
+      <c r="G14" s="46" t="inlineStr">
         <is>
           <t>Building is safe to occupy; snag list issued.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1">
-      <c r="B15" s="34" t="inlineStr">
+      <c r="B15" s="41" t="inlineStr">
         <is>
           <t>M09</t>
         </is>
       </c>
-      <c r="C15" s="35" t="inlineStr">
+      <c r="C15" s="42" t="inlineStr">
         <is>
           <t>Handover to client</t>
         </is>
       </c>
-      <c r="D15" s="36" t="inlineStr">
+      <c r="D15" s="43" t="inlineStr">
         <is>
           <t>25 Sep 2026</t>
         </is>
       </c>
-      <c r="E15" s="41" t="inlineStr">
+      <c r="E15" s="48" t="inlineStr">
         <is>
           <t>On track</t>
         </is>
       </c>
-      <c r="F15" s="38" t="inlineStr">
+      <c r="F15" s="45" t="inlineStr">
         <is>
           <t>PM</t>
         </is>
       </c>
-      <c r="G15" s="39" t="inlineStr">
+      <c r="G15" s="46" t="inlineStr">
         <is>
           <t>All snags cleared, documentation and warranties transferred.</t>
         </is>
@@ -2089,34 +2453,34 @@
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="42" t="inlineStr">
+      <c r="B6" s="49" t="inlineStr">
         <is>
           <t>SCOPE</t>
         </is>
       </c>
-      <c r="C6" s="42" t="inlineStr">
+      <c r="C6" s="49" t="inlineStr">
         <is>
           <t>REF</t>
         </is>
       </c>
-      <c r="D6" s="42" t="inlineStr">
+      <c r="D6" s="49" t="inlineStr">
         <is>
           <t>REASON</t>
         </is>
       </c>
     </row>
     <row r="7" ht="54" customHeight="1">
-      <c r="B7" s="43" t="inlineStr">
+      <c r="B7" s="50" t="inlineStr">
         <is>
           <t>milestones</t>
         </is>
       </c>
-      <c r="C7" s="26" t="inlineStr">
+      <c r="C7" s="25" t="inlineStr">
         <is>
           <t>M03</t>
         </is>
       </c>
-      <c r="D7" s="44" t="inlineStr">
+      <c r="D7" s="51" t="inlineStr">
         <is>
           <t>Permit sign-off is trending five working days behind the internal target. Recommend the client clears a pre-meeting slot with the city permits office in the next ten days to de-risk the 30 April date.</t>
         </is>

</xml_diff>